<commit_message>
Methods from cited papers; declare dependencies
- harmonize/papers.py: plan (cited works of packages with an unknown method, OpenAlex lookup, plan.csv), download (approved rows only, into data/source/papers/), status.
- method_for: paper text as the last method source, only in the clause naming the variable.
- pyproject.toml: [project] with the dependencies (pandas below 3, as the outputs were made with 2.3).
- Soil pH and Total carbon outputs: 10.15485/1960313 pH_H2O and dry_combustion, 10.15485/1631979 dry_combustion.
</commit_message>
<xml_diff>
--- a/data/processed/harmonization/Acidity__Soil_pH/10.15485_1960313/10.15485_1960313_soil_Acidity__Soil_pH.xlsx
+++ b/data/processed/harmonization/Acidity__Soil_pH/10.15485_1960313/10.15485_1960313_soil_Acidity__Soil_pH.xlsx
@@ -537,7 +537,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -553,7 +553,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -605,7 +605,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -657,7 +657,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -709,7 +709,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -761,7 +761,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -813,7 +813,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -849,7 +849,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -865,7 +865,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -917,7 +917,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -953,7 +953,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -969,7 +969,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1005,7 +1005,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1213,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I16" t="n">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I17" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I18" t="n">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I19" t="n">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1473,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I20" t="n">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1525,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I21" t="n">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1577,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I22" t="n">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1629,7 +1629,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I23" t="n">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I24" t="n">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I25" t="n">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1785,7 +1785,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I26" t="n">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1837,7 +1837,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I27" t="n">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1889,7 +1889,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I28" t="n">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I29" t="n">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -1993,7 +1993,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I30" t="n">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I31" t="n">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I32" t="n">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2149,7 +2149,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I33" t="n">
@@ -2165,7 +2165,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I34" t="n">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2253,7 +2253,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I35" t="n">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2305,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I36" t="n">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2357,7 +2357,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I37" t="n">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I38" t="n">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I39" t="n">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I40" t="n">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2565,7 +2565,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I41" t="n">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I42" t="n">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2669,7 +2669,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I43" t="n">
@@ -2685,7 +2685,7 @@
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I44" t="n">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I45" t="n">
@@ -2789,7 +2789,7 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2825,7 +2825,7 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I46" t="n">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2877,7 +2877,7 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I47" t="n">
@@ -2893,7 +2893,7 @@
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2929,7 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I48" t="n">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2981,7 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I49" t="n">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I50" t="n">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3085,7 +3085,7 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I51" t="n">
@@ -3101,7 +3101,7 @@
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I52" t="n">
@@ -3153,7 +3153,7 @@
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3189,7 +3189,7 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I53" t="n">
@@ -3205,7 +3205,7 @@
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I54" t="n">
@@ -3257,7 +3257,7 @@
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3293,7 +3293,7 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I55" t="n">
@@ -3309,7 +3309,7 @@
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I56" t="n">
@@ -3361,7 +3361,7 @@
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I57" t="n">
@@ -3413,7 +3413,7 @@
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3449,7 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I58" t="n">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I59" t="n">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3553,7 +3553,7 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I60" t="n">
@@ -3569,7 +3569,7 @@
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I61" t="n">
@@ -3621,7 +3621,7 @@
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3657,7 +3657,7 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I62" t="n">
@@ -3673,7 +3673,7 @@
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3709,7 +3709,7 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I63" t="n">
@@ -3725,7 +3725,7 @@
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I64" t="n">
@@ -3777,7 +3777,7 @@
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3813,7 +3813,7 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I65" t="n">
@@ -3829,7 +3829,7 @@
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3865,7 +3865,7 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I66" t="n">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3917,7 +3917,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I67" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -3969,7 +3969,7 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I68" t="n">
@@ -3985,7 +3985,7 @@
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4021,7 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I69" t="n">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4073,7 +4073,7 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I70" t="n">
@@ -4089,7 +4089,7 @@
       </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I71" t="n">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4177,7 +4177,7 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I72" t="n">
@@ -4193,7 +4193,7 @@
       </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4229,7 +4229,7 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I73" t="n">
@@ -4245,7 +4245,7 @@
       </c>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I74" t="n">
@@ -4297,7 +4297,7 @@
       </c>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4333,7 +4333,7 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I75" t="n">
@@ -4349,7 +4349,7 @@
       </c>
       <c r="L75" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4385,7 +4385,7 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I76" t="n">
@@ -4401,7 +4401,7 @@
       </c>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4437,7 +4437,7 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I77" t="n">
@@ -4453,7 +4453,7 @@
       </c>
       <c r="L77" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4489,7 +4489,7 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I78" t="n">
@@ -4505,7 +4505,7 @@
       </c>
       <c r="L78" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4541,7 +4541,7 @@
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I79" t="n">
@@ -4557,7 +4557,7 @@
       </c>
       <c r="L79" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4593,7 +4593,7 @@
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I80" t="n">
@@ -4609,7 +4609,7 @@
       </c>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4645,7 +4645,7 @@
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I81" t="n">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4697,7 +4697,7 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I82" t="n">
@@ -4713,7 +4713,7 @@
       </c>
       <c r="L82" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4749,7 +4749,7 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I83" t="n">
@@ -4765,7 +4765,7 @@
       </c>
       <c r="L83" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4801,7 +4801,7 @@
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I84" t="n">
@@ -4817,7 +4817,7 @@
       </c>
       <c r="L84" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4853,7 +4853,7 @@
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I85" t="n">
@@ -4869,7 +4869,7 @@
       </c>
       <c r="L85" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4905,7 +4905,7 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I86" t="n">
@@ -4921,7 +4921,7 @@
       </c>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4957,7 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I87" t="n">
@@ -4973,7 +4973,7 @@
       </c>
       <c r="L87" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5009,7 +5009,7 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I88" t="n">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="L88" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5061,7 +5061,7 @@
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I89" t="n">
@@ -5077,7 +5077,7 @@
       </c>
       <c r="L89" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5113,7 +5113,7 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I90" t="n">
@@ -5129,7 +5129,7 @@
       </c>
       <c r="L90" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5165,7 +5165,7 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I91" t="n">
@@ -5181,7 +5181,7 @@
       </c>
       <c r="L91" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I92" t="n">
@@ -5233,7 +5233,7 @@
       </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5269,7 +5269,7 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I93" t="n">
@@ -5285,7 +5285,7 @@
       </c>
       <c r="L93" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5321,7 +5321,7 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I94" t="n">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5373,7 +5373,7 @@
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I95" t="n">
@@ -5389,7 +5389,7 @@
       </c>
       <c r="L95" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5425,7 +5425,7 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I96" t="n">
@@ -5441,7 +5441,7 @@
       </c>
       <c r="L96" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5477,7 +5477,7 @@
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I97" t="n">
@@ -5493,7 +5493,7 @@
       </c>
       <c r="L97" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5529,7 +5529,7 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I98" t="n">
@@ -5545,7 +5545,7 @@
       </c>
       <c r="L98" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5581,7 +5581,7 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I99" t="n">
@@ -5597,7 +5597,7 @@
       </c>
       <c r="L99" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5633,7 +5633,7 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I100" t="n">
@@ -5649,7 +5649,7 @@
       </c>
       <c r="L100" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5685,7 +5685,7 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I101" t="n">
@@ -5701,7 +5701,7 @@
       </c>
       <c r="L101" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5737,7 +5737,7 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I102" t="n">
@@ -5753,7 +5753,7 @@
       </c>
       <c r="L102" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5789,7 +5789,7 @@
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I103" t="n">
@@ -5805,7 +5805,7 @@
       </c>
       <c r="L103" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5841,7 +5841,7 @@
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I104" t="n">
@@ -5857,7 +5857,7 @@
       </c>
       <c r="L104" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5893,7 +5893,7 @@
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I105" t="n">
@@ -5909,7 +5909,7 @@
       </c>
       <c r="L105" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5945,7 +5945,7 @@
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I106" t="n">
@@ -5961,7 +5961,7 @@
       </c>
       <c r="L106" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I107" t="n">
@@ -6013,7 +6013,7 @@
       </c>
       <c r="L107" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6049,7 +6049,7 @@
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I108" t="n">
@@ -6065,7 +6065,7 @@
       </c>
       <c r="L108" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6101,7 +6101,7 @@
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I109" t="n">
@@ -6117,7 +6117,7 @@
       </c>
       <c r="L109" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6153,7 +6153,7 @@
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I110" t="n">
@@ -6169,7 +6169,7 @@
       </c>
       <c r="L110" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6205,7 +6205,7 @@
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I111" t="n">
@@ -6221,7 +6221,7 @@
       </c>
       <c r="L111" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6257,7 +6257,7 @@
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I112" t="n">
@@ -6273,7 +6273,7 @@
       </c>
       <c r="L112" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I113" t="n">
@@ -6325,7 +6325,7 @@
       </c>
       <c r="L113" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6361,7 +6361,7 @@
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I114" t="n">
@@ -6377,7 +6377,7 @@
       </c>
       <c r="L114" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6413,7 +6413,7 @@
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I115" t="n">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="L115" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6465,7 +6465,7 @@
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I116" t="n">
@@ -6481,7 +6481,7 @@
       </c>
       <c r="L116" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6517,7 +6517,7 @@
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I117" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="L117" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6569,7 +6569,7 @@
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I118" t="n">
@@ -6585,7 +6585,7 @@
       </c>
       <c r="L118" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6621,7 +6621,7 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I119" t="n">
@@ -6637,7 +6637,7 @@
       </c>
       <c r="L119" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6673,7 +6673,7 @@
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I120" t="n">
@@ -6689,7 +6689,7 @@
       </c>
       <c r="L120" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6725,7 +6725,7 @@
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I121" t="n">
@@ -6741,7 +6741,7 @@
       </c>
       <c r="L121" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6777,7 +6777,7 @@
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I122" t="n">
@@ -6793,7 +6793,7 @@
       </c>
       <c r="L122" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6829,7 +6829,7 @@
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I123" t="n">
@@ -6845,7 +6845,7 @@
       </c>
       <c r="L123" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6881,7 +6881,7 @@
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I124" t="n">
@@ -6897,7 +6897,7 @@
       </c>
       <c r="L124" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I125" t="n">
@@ -6949,7 +6949,7 @@
       </c>
       <c r="L125" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -6985,7 +6985,7 @@
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I126" t="n">
@@ -7001,7 +7001,7 @@
       </c>
       <c r="L126" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7037,7 +7037,7 @@
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I127" t="n">
@@ -7053,7 +7053,7 @@
       </c>
       <c r="L127" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7089,7 +7089,7 @@
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I128" t="n">
@@ -7105,7 +7105,7 @@
       </c>
       <c r="L128" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7141,7 +7141,7 @@
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I129" t="n">
@@ -7157,7 +7157,7 @@
       </c>
       <c r="L129" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7193,7 +7193,7 @@
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I130" t="n">
@@ -7209,7 +7209,7 @@
       </c>
       <c r="L130" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7245,7 +7245,7 @@
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I131" t="n">
@@ -7261,7 +7261,7 @@
       </c>
       <c r="L131" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7297,7 +7297,7 @@
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I132" t="n">
@@ -7313,7 +7313,7 @@
       </c>
       <c r="L132" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7349,7 +7349,7 @@
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I133" t="n">
@@ -7365,7 +7365,7 @@
       </c>
       <c r="L133" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7401,7 +7401,7 @@
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I134" t="n">
@@ -7417,7 +7417,7 @@
       </c>
       <c r="L134" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7453,7 +7453,7 @@
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I135" t="n">
@@ -7469,7 +7469,7 @@
       </c>
       <c r="L135" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7505,7 +7505,7 @@
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I136" t="n">
@@ -7521,7 +7521,7 @@
       </c>
       <c r="L136" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7557,7 +7557,7 @@
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I137" t="n">
@@ -7573,7 +7573,7 @@
       </c>
       <c r="L137" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7609,7 +7609,7 @@
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I138" t="n">
@@ -7625,7 +7625,7 @@
       </c>
       <c r="L138" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7661,7 +7661,7 @@
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I139" t="n">
@@ -7677,7 +7677,7 @@
       </c>
       <c r="L139" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7713,7 +7713,7 @@
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I140" t="n">
@@ -7729,7 +7729,7 @@
       </c>
       <c r="L140" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7765,7 +7765,7 @@
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I141" t="n">
@@ -7781,7 +7781,7 @@
       </c>
       <c r="L141" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7817,7 +7817,7 @@
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I142" t="n">
@@ -7833,7 +7833,7 @@
       </c>
       <c r="L142" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7869,7 +7869,7 @@
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I143" t="n">
@@ -7885,7 +7885,7 @@
       </c>
       <c r="L143" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7921,7 +7921,7 @@
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I144" t="n">
@@ -7937,7 +7937,7 @@
       </c>
       <c r="L144" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -7973,7 +7973,7 @@
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I145" t="n">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="L145" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8025,7 +8025,7 @@
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I146" t="n">
@@ -8041,7 +8041,7 @@
       </c>
       <c r="L146" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8077,7 +8077,7 @@
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I147" t="n">
@@ -8093,7 +8093,7 @@
       </c>
       <c r="L147" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8129,7 +8129,7 @@
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I148" t="n">
@@ -8145,7 +8145,7 @@
       </c>
       <c r="L148" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8181,7 +8181,7 @@
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I149" t="n">
@@ -8197,7 +8197,7 @@
       </c>
       <c r="L149" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8233,7 +8233,7 @@
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I150" t="n">
@@ -8249,7 +8249,7 @@
       </c>
       <c r="L150" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8285,7 +8285,7 @@
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I151" t="n">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="L151" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8337,7 +8337,7 @@
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I152" t="n">
@@ -8353,7 +8353,7 @@
       </c>
       <c r="L152" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8389,7 +8389,7 @@
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I153" t="n">
@@ -8405,7 +8405,7 @@
       </c>
       <c r="L153" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I154" t="n">
@@ -8457,7 +8457,7 @@
       </c>
       <c r="L154" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8493,7 +8493,7 @@
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I155" t="n">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="L155" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8545,7 +8545,7 @@
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I156" t="n">
@@ -8561,7 +8561,7 @@
       </c>
       <c r="L156" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8597,7 +8597,7 @@
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I157" t="n">
@@ -8613,7 +8613,7 @@
       </c>
       <c r="L157" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8649,7 +8649,7 @@
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I158" t="n">
@@ -8665,7 +8665,7 @@
       </c>
       <c r="L158" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8701,7 +8701,7 @@
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I159" t="n">
@@ -8717,7 +8717,7 @@
       </c>
       <c r="L159" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8753,7 +8753,7 @@
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I160" t="n">
@@ -8769,7 +8769,7 @@
       </c>
       <c r="L160" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8805,7 +8805,7 @@
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I161" t="n">
@@ -8821,7 +8821,7 @@
       </c>
       <c r="L161" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8857,7 +8857,7 @@
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I162" t="n">
@@ -8873,7 +8873,7 @@
       </c>
       <c r="L162" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8909,7 +8909,7 @@
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I163" t="n">
@@ -8925,7 +8925,7 @@
       </c>
       <c r="L163" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -8961,7 +8961,7 @@
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I164" t="n">
@@ -8977,7 +8977,7 @@
       </c>
       <c r="L164" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -9013,7 +9013,7 @@
       </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I165" t="n">
@@ -9029,7 +9029,7 @@
       </c>
       <c r="L165" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -9065,7 +9065,7 @@
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I166" t="n">
@@ -9081,7 +9081,7 @@
       </c>
       <c r="L166" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -9117,7 +9117,7 @@
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I167" t="n">
@@ -9133,7 +9133,7 @@
       </c>
       <c r="L167" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -9169,7 +9169,7 @@
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I168" t="n">
@@ -9185,7 +9185,7 @@
       </c>
       <c r="L168" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -9221,7 +9221,7 @@
       </c>
       <c r="H169" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I169" t="n">
@@ -9237,7 +9237,7 @@
       </c>
       <c r="L169" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -9273,7 +9273,7 @@
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I170" t="n">
@@ -9289,7 +9289,7 @@
       </c>
       <c r="L170" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -9325,7 +9325,7 @@
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I171" t="n">
@@ -9341,7 +9341,7 @@
       </c>
       <c r="L171" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -9377,7 +9377,7 @@
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I172" t="n">
@@ -9393,7 +9393,7 @@
       </c>
       <c r="L172" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -9429,7 +9429,7 @@
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I173" t="n">
@@ -9445,7 +9445,7 @@
       </c>
       <c r="L173" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -9481,7 +9481,7 @@
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I174" t="n">
@@ -9497,7 +9497,7 @@
       </c>
       <c r="L174" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -9533,7 +9533,7 @@
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I175" t="n">
@@ -9549,7 +9549,7 @@
       </c>
       <c r="L175" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -9585,7 +9585,7 @@
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I176" t="n">
@@ -9601,7 +9601,7 @@
       </c>
       <c r="L176" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -9637,7 +9637,7 @@
       </c>
       <c r="H177" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I177" t="n">
@@ -9653,7 +9653,7 @@
       </c>
       <c r="L177" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -9689,7 +9689,7 @@
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I178" t="n">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="L178" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -9741,7 +9741,7 @@
       </c>
       <c r="H179" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I179" t="n">
@@ -9757,7 +9757,7 @@
       </c>
       <c r="L179" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>
@@ -9793,7 +9793,7 @@
       </c>
       <c r="H180" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>pH_H2O</t>
         </is>
       </c>
       <c r="I180" t="n">
@@ -9809,7 +9809,7 @@
       </c>
       <c r="L180" s="2" t="inlineStr">
         <is>
-          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage</t>
+          <t>lat/long source: doi:10.15485/1960313 package spatialCoverage named point; data key kit_id; source column ph; date 2021 from package temporal coverage; method from cited paper doi:10.1038/s41597-023-02548-7</t>
         </is>
       </c>
     </row>

</xml_diff>